<commit_message>
Oppdater stats – ny spiller lagt til
</commit_message>
<xml_diff>
--- a/CS_Stats_Komplettligaen Counter-strike - Våren 20.xlsx
+++ b/CS_Stats_Komplettligaen Counter-strike - Våren 20.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stats" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Stats" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,12 +46,12 @@
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="0000FF88"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00FFFFFF"/>
+      <b val="1"/>
+      <color rgb="0000FF88"/>
       <sz val="10"/>
     </font>
     <font>
@@ -130,31 +130,31 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -651,52 +651,52 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>81</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>18</v>
+        <v>261</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>23</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>108</v>
+        <v>320</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>10259</v>
+        <v>1.08</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>27094</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>61</v>
+        <v>36</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>50</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="N3" s="7" t="n">
-        <v>30</v>
+        <v>56</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>26</v>
       </c>
       <c r="O3" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="P3" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="P3" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q3" s="4" t="n">
-        <v>1</v>
+      <c r="Q3" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="R3" s="4" t="n">
         <v>0</v>
@@ -709,54 +709,54 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>85</v>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>29</v>
+        <v>240</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>75</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>86</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F4" s="10" t="n">
-        <v>108</v>
+        <v>248</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>320</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>9103</v>
+        <v>26112</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="L4" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="M4" s="10" t="n">
-        <v>20</v>
+        <v>5</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>48</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="R4" s="11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -766,53 +766,53 @@
           <t>Waffuru</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>71</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>87</v>
+      <c r="B5" s="5" t="n">
+        <v>229</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>247</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>-16</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>107</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>0.87</v>
+        <v>-18</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>320</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.96</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>8070</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>74</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>37</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="M5" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="O5" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q5" s="4" t="n">
-        <v>1</v>
+        <v>26795</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="R5" s="4" t="n">
         <v>0</v>
@@ -821,58 +821,58 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Gru91</t>
+          <t>woznor</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>81</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>-30</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>108</v>
+        <v>12</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>-4</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>70</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.67</v>
+        <v>0.89</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>6297</v>
+        <v>4850</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="J6" s="9" t="n">
         <v>7</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -882,55 +882,171 @@
           <t>MarcusCraig</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>52</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>87</v>
+      <c r="B7" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>252</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>-35</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>107</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>0.64</v>
+        <v>-62</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>320</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>5803</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>53</v>
-      </c>
-      <c r="J7" s="7" t="n">
+        <v>20872</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="P7" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="Q7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Gru91</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>156</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>-63</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>203</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>11360</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="K8" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="L7" s="7" t="n">
+      <c r="L8" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="P8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="M7" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="O7" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="P7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q7" s="7" t="n">
+      <c r="R8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="R7" s="4" t="n">
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>NinjaDaniel</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>-22</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>1917</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>